<commit_message>
fix(core): when an end has no neighbouring holes, push the chain ends 3m along strike instead of closing with a through-line (keeps P1/P2 inside)
</commit_message>
<xml_diff>
--- a/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008_strip/3940平台 1008炮孔数据报告.xlsx
+++ b/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008_strip/3940平台 1008炮孔数据报告.xlsx
@@ -521,16 +521,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>1544.903</v>
+        <v>1571.642</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>4171.237</v>
+        <v>4243.433</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>1.204</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>50.236</v>
+        <v>51.106</v>
       </c>
     </row>
     <row r="4">
@@ -541,16 +541,16 @@
       </c>
       <c r="B4" s="6" t="n"/>
       <c r="C4" s="7" t="n">
-        <v>1544.903</v>
+        <v>1571.642</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>4171.237</v>
+        <v>4243.433</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>1.204</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>50.236</v>
+        <v>51.106</v>
       </c>
     </row>
     <row r="5">
@@ -625,16 +625,16 @@
       </c>
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="9" t="n">
-        <v>3681.486</v>
+        <v>3708.226</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>9940.012000000001</v>
+        <v>10012.209</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>0.917</v>
+        <v>0.919</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>91.17100000000001</v>
+        <v>92.04000000000001</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
feat(core): outline = ore-hole Voronoi cells clipped to all-hole hull + 3m (midpoint to neighbours inside, 3m outwards where no holes)
</commit_message>
<xml_diff>
--- a/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008_strip/3940平台 1008炮孔数据报告.xlsx
+++ b/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008_strip/3940平台 1008炮孔数据报告.xlsx
@@ -521,16 +521,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>1571.642</v>
+        <v>2098.075</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>4243.433</v>
+        <v>5664.802</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>1.204</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>51.106</v>
+        <v>68.224</v>
       </c>
     </row>
     <row r="4">
@@ -541,16 +541,16 @@
       </c>
       <c r="B4" s="6" t="n"/>
       <c r="C4" s="7" t="n">
-        <v>1571.642</v>
+        <v>2098.075</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>4243.433</v>
+        <v>5664.802</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>1.204</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>51.106</v>
+        <v>68.224</v>
       </c>
     </row>
     <row r="5">
@@ -563,16 +563,16 @@
         <v>2</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>1286.594</v>
+        <v>2064.946</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>3473.804</v>
+        <v>5575.355</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>0.729</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>25.329</v>
+        <v>40.652</v>
       </c>
     </row>
     <row r="6">
@@ -585,16 +585,16 @@
         <v>3</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>849.989</v>
+        <v>767.37</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>2294.971</v>
+        <v>2071.9</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>0.68</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>15.606</v>
+        <v>14.089</v>
       </c>
     </row>
     <row r="7">
@@ -605,16 +605,16 @@
       </c>
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="7" t="n">
-        <v>2136.584</v>
+        <v>2832.317</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>5768.776</v>
+        <v>7647.255</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.71</v>
+        <v>0.716</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>40.934</v>
+        <v>54.741</v>
       </c>
     </row>
     <row r="8">
@@ -625,16 +625,16 @@
       </c>
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="9" t="n">
-        <v>3708.226</v>
+        <v>4930.391</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>10012.209</v>
+        <v>13312.057</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>0.919</v>
+        <v>0.924</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>92.04000000000001</v>
+        <v>122.964</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
feat(core): simplify zone outline (tolerance 0.8m, configurable) so boundaries stay straight with few vertices
</commit_message>
<xml_diff>
--- a/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008_strip/3940平台 1008炮孔数据报告.xlsx
+++ b/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008_strip/3940平台 1008炮孔数据报告.xlsx
@@ -521,16 +521,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>2098.075</v>
+        <v>2096.144</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>5664.802</v>
+        <v>5659.588</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>1.204</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>68.224</v>
+        <v>68.161</v>
       </c>
     </row>
     <row r="4">
@@ -541,16 +541,16 @@
       </c>
       <c r="B4" s="6" t="n"/>
       <c r="C4" s="7" t="n">
-        <v>2098.075</v>
+        <v>2096.144</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>5664.802</v>
+        <v>5659.588</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>1.204</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>68.224</v>
+        <v>68.161</v>
       </c>
     </row>
     <row r="5">
@@ -563,16 +563,16 @@
         <v>2</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>2064.946</v>
+        <v>2063.183</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>5575.355</v>
+        <v>5570.593</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>0.729</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>40.652</v>
+        <v>40.617</v>
       </c>
     </row>
     <row r="6">
@@ -585,16 +585,16 @@
         <v>3</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>767.37</v>
+        <v>765.178</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>2071.9</v>
+        <v>2065.982</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>0.68</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>14.089</v>
+        <v>14.049</v>
       </c>
     </row>
     <row r="7">
@@ -605,16 +605,16 @@
       </c>
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="7" t="n">
-        <v>2832.317</v>
+        <v>2828.361</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>7647.255</v>
+        <v>7636.574</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>0.716</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>54.741</v>
+        <v>54.666</v>
       </c>
     </row>
     <row r="8">
@@ -625,16 +625,16 @@
       </c>
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="9" t="n">
-        <v>4930.391</v>
+        <v>4924.505</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>13312.057</v>
+        <v>13296.163</v>
       </c>
       <c r="E8" s="9" t="n">
         <v>0.924</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>122.964</v>
+        <v>122.827</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
core: zone outline back to chain-polyline structure (matches manual drawing's vertex count) + simplify; end-closure selection still needs refinement
</commit_message>
<xml_diff>
--- a/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008_strip/3940平台 1008炮孔数据报告.xlsx
+++ b/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008_strip/3940平台 1008炮孔数据报告.xlsx
@@ -521,16 +521,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>2096.144</v>
+        <v>1503.976</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>5659.588</v>
+        <v>4060.734</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>1.204</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>68.161</v>
+        <v>48.905</v>
       </c>
     </row>
     <row r="4">
@@ -541,16 +541,16 @@
       </c>
       <c r="B4" s="6" t="n"/>
       <c r="C4" s="7" t="n">
-        <v>2096.144</v>
+        <v>1503.976</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>5659.588</v>
+        <v>4060.734</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>1.204</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>68.161</v>
+        <v>48.905</v>
       </c>
     </row>
     <row r="5">
@@ -563,16 +563,16 @@
         <v>2</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>2063.183</v>
+        <v>869.164</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>5570.593</v>
+        <v>2346.742</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>0.729</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>40.617</v>
+        <v>17.111</v>
       </c>
     </row>
     <row r="6">
@@ -585,16 +585,16 @@
         <v>3</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>765.178</v>
+        <v>392.403</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>2065.982</v>
+        <v>1059.487</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>0.68</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>14.049</v>
+        <v>7.205</v>
       </c>
     </row>
     <row r="7">
@@ -605,16 +605,16 @@
       </c>
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="7" t="n">
-        <v>2828.361</v>
+        <v>1261.566</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>7636.574</v>
+        <v>3406.229</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.716</v>
+        <v>0.714</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>54.666</v>
+        <v>24.315</v>
       </c>
     </row>
     <row r="8">
@@ -625,16 +625,16 @@
       </c>
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="9" t="n">
-        <v>4924.505</v>
+        <v>2765.542</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>13296.163</v>
+        <v>7466.963</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>0.924</v>
+        <v>0.981</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>122.827</v>
+        <v>73.221</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
chore: regenerate 1008 deliverables with rule-driven grade lines and end-band midpoint chains
</commit_message>
<xml_diff>
--- a/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008_strip/3940平台 1008炮孔数据报告.xlsx
+++ b/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008_strip/3940平台 1008炮孔数据报告.xlsx
@@ -521,16 +521,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>1503.976</v>
+        <v>1451.784</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>4060.734</v>
+        <v>3919.818</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>1.204</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>48.905</v>
+        <v>47.208</v>
       </c>
     </row>
     <row r="4">
@@ -541,16 +541,16 @@
       </c>
       <c r="B4" s="6" t="n"/>
       <c r="C4" s="7" t="n">
-        <v>1503.976</v>
+        <v>1451.784</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>4060.734</v>
+        <v>3919.818</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>1.204</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>48.905</v>
+        <v>47.208</v>
       </c>
     </row>
     <row r="5">
@@ -563,16 +563,16 @@
         <v>2</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>869.164</v>
+        <v>1274.185</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>2346.742</v>
+        <v>3440.301</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>0.729</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>17.111</v>
+        <v>25.084</v>
       </c>
     </row>
     <row r="6">
@@ -585,16 +585,16 @@
         <v>3</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>392.403</v>
+        <v>816.062</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>1059.487</v>
+        <v>2203.368</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>0.68</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>7.205</v>
+        <v>14.983</v>
       </c>
     </row>
     <row r="7">
@@ -605,16 +605,16 @@
       </c>
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="7" t="n">
-        <v>1261.566</v>
+        <v>2090.247</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>3406.229</v>
+        <v>5643.668</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.714</v>
+        <v>0.71</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>24.315</v>
+        <v>40.067</v>
       </c>
     </row>
     <row r="8">
@@ -625,16 +625,16 @@
       </c>
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="9" t="n">
-        <v>2765.542</v>
+        <v>3542.032</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>7466.963</v>
+        <v>9563.486000000001</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>0.981</v>
+        <v>0.913</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>73.221</v>
+        <v>87.27500000000001</v>
       </c>
     </row>
     <row r="9">

</xml_diff>